<commit_message>
Cambios para añadir nuevas integraciones
</commit_message>
<xml_diff>
--- a/Resultado_Inventario.xlsx
+++ b/Resultado_Inventario.xlsx
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="13">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="14">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29">
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">

</xml_diff>

<commit_message>
Cambios para agregar nueva funcion
</commit_message>
<xml_diff>
--- a/Resultado_Inventario.xlsx
+++ b/Resultado_Inventario.xlsx
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">

</xml_diff>